<commit_message>
fix(contract-bundle): contract serial no, paid options rows, asset sheet iteration & safety sheet assetNo only (v2.0.0.Build.20)
</commit_message>
<xml_diff>
--- a/public/03.안전점검결과서.xlsx
+++ b/public/03.안전점검결과서.xlsx
@@ -5,19 +5,16 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\OneDrive\Desktop\기연리프트자료_\261016_최종업로드\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\eBroAgent\drive_mirror\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{53CC7E3C-0660-46E1-96D6-E7B47AA65EA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A44DFA44-D305-462E-8C1D-5F19685050F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D8DB1586-3BC3-454B-8B50-94F91773DC5F}"/>
   </bookViews>
   <sheets>
     <sheet name="안전점검결과서" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="동력">#REF!</definedName>
     <definedName name="등판능력">#REF!</definedName>
@@ -132,10 +129,6 @@
     <t>차량번호</t>
   </si>
   <si>
-    <t>{차량번호}</t>
-    <phoneticPr fontId="3" type="noConversion"/>
-  </si>
-  <si>
     <t>제조년도</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
@@ -360,6 +353,10 @@
   </si>
   <si>
     <t>검사자 의견</t>
+  </si>
+  <si>
+    <t>{관리번호}</t>
+    <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -621,95 +618,95 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -948,26 +945,6 @@
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="계약서 "/>
-      <sheetName val="반입전체크리스트"/>
-      <sheetName val="안전점검결과서"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1305,73 +1282,73 @@
       <c r="B3" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="5"/>
+      <c r="D3" s="29"/>
       <c r="E3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="8"/>
-      <c r="I3" s="9" t="s">
+      <c r="H3" s="26"/>
+      <c r="I3" s="31" t="s">
         <v>5</v>
       </c>
-      <c r="J3" s="10"/>
-      <c r="K3" s="11"/>
+      <c r="J3" s="34"/>
+      <c r="K3" s="32"/>
     </row>
     <row r="4" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="9" t="s">
+      <c r="C4" s="31" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="11"/>
+      <c r="D4" s="32"/>
       <c r="E4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="F4" s="6" t="s">
+      <c r="F4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="H4" s="8"/>
-      <c r="I4" s="4" t="s">
+      <c r="H4" s="26"/>
+      <c r="I4" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="J4" s="12"/>
-      <c r="K4" s="5"/>
+      <c r="J4" s="28"/>
+      <c r="K4" s="29"/>
     </row>
     <row r="5" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="27" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="5"/>
+      <c r="D5" s="29"/>
       <c r="E5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="F5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="25" t="s">
         <v>16</v>
       </c>
-      <c r="H5" s="8"/>
-      <c r="I5" s="4" t="s">
+      <c r="H5" s="26"/>
+      <c r="I5" s="27" t="s">
         <v>17</v>
       </c>
-      <c r="J5" s="5"/>
-      <c r="K5" s="6" t="s">
+      <c r="J5" s="29"/>
+      <c r="K5" s="5" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1379,635 +1356,635 @@
       <c r="B6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C6" s="9" t="s">
+      <c r="C6" s="31" t="s">
+        <v>86</v>
+      </c>
+      <c r="D6" s="32"/>
+      <c r="E6" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="3" t="s">
+      <c r="F6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="6" t="s">
+      <c r="G6" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="H6" s="26"/>
+      <c r="I6" s="33" t="s">
         <v>23</v>
       </c>
-      <c r="H6" s="8"/>
-      <c r="I6" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="J6" s="12"/>
-      <c r="K6" s="5"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="29"/>
     </row>
     <row r="7" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="D7" s="24"/>
+      <c r="E7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="F7" s="16" t="s">
+      <c r="G7" s="25" t="s">
         <v>28</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="H7" s="26"/>
+      <c r="I7" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="J7" s="12"/>
-      <c r="K7" s="5"/>
+      <c r="J7" s="28"/>
+      <c r="K7" s="29"/>
     </row>
     <row r="8" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B8" s="17"/>
-      <c r="C8" s="18"/>
-      <c r="D8" s="18"/>
-      <c r="E8" s="18"/>
-      <c r="F8" s="18"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="18"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="19"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="10"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" s="25" t="s">
         <v>31</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="30"/>
+      <c r="E9" s="30"/>
+      <c r="F9" s="30"/>
+      <c r="G9" s="30"/>
+      <c r="H9" s="26"/>
+      <c r="I9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
-      <c r="H9" s="8"/>
-      <c r="I9" s="3" t="s">
+      <c r="J9" s="25" t="s">
         <v>33</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="K9" s="26"/>
+    </row>
+    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B10" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="K9" s="8"/>
-    </row>
-    <row r="10" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B10" s="17" t="s">
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="10"/>
+    </row>
+    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B11" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="18"/>
-      <c r="D10" s="18"/>
-      <c r="E10" s="18"/>
-      <c r="F10" s="18"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="18"/>
-      <c r="J10" s="18"/>
-      <c r="K10" s="19"/>
-    </row>
-    <row r="11" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B11" s="21" t="s">
+      <c r="C11" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="17" t="s">
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="19"/>
-      <c r="I11" s="6" t="s">
+      <c r="J11" s="8"/>
+      <c r="K11" s="10"/>
+    </row>
+    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B12" s="12"/>
+      <c r="C12" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="J11" s="17"/>
-      <c r="K11" s="19"/>
-    </row>
-    <row r="12" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B12" s="22"/>
-      <c r="C12" s="17" t="s">
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="18"/>
-      <c r="E12" s="18"/>
-      <c r="F12" s="18"/>
-      <c r="G12" s="18"/>
-      <c r="H12" s="19"/>
-      <c r="I12" s="6" t="s">
+      <c r="J12" s="8"/>
+      <c r="K12" s="10"/>
+    </row>
+    <row r="13" spans="2:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="13"/>
+      <c r="C13" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="17"/>
-      <c r="K12" s="19"/>
-    </row>
-    <row r="13" spans="2:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="23"/>
-      <c r="C13" s="17" t="s">
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J13" s="8"/>
+      <c r="K13" s="10"/>
+    </row>
+    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B14" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="19"/>
-      <c r="I13" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J13" s="17"/>
-      <c r="K13" s="19"/>
-    </row>
-    <row r="14" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B14" s="17" t="s">
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="10"/>
+    </row>
+    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B15" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="C14" s="18"/>
-      <c r="D14" s="18"/>
-      <c r="E14" s="18"/>
-      <c r="F14" s="18"/>
-      <c r="G14" s="18"/>
-      <c r="H14" s="18"/>
-      <c r="I14" s="18"/>
-      <c r="J14" s="18"/>
-      <c r="K14" s="19"/>
-    </row>
-    <row r="15" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B15" s="21" t="s">
+      <c r="C15" s="8" t="s">
         <v>43</v>
       </c>
-      <c r="C15" s="17" t="s">
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J15" s="17"/>
+      <c r="K15" s="18"/>
+    </row>
+    <row r="16" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="13"/>
+      <c r="C16" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="D15" s="18"/>
-      <c r="E15" s="18"/>
-      <c r="F15" s="18"/>
-      <c r="G15" s="18"/>
-      <c r="H15" s="19"/>
-      <c r="I15" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J15" s="25"/>
-      <c r="K15" s="26"/>
-    </row>
-    <row r="16" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B16" s="23"/>
-      <c r="C16" s="17" t="s">
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="21"/>
+      <c r="K16" s="22"/>
+    </row>
+    <row r="17" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="D16" s="18"/>
-      <c r="E16" s="18"/>
-      <c r="F16" s="18"/>
-      <c r="G16" s="18"/>
-      <c r="H16" s="19"/>
-      <c r="I16" s="27"/>
-      <c r="J16" s="28"/>
-      <c r="K16" s="29"/>
-    </row>
-    <row r="17" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B17" s="21" t="s">
+      <c r="C17" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="17" t="s">
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J17" s="17"/>
+      <c r="K17" s="18"/>
+    </row>
+    <row r="18" spans="2:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="12"/>
+      <c r="C18" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="18"/>
-      <c r="E17" s="18"/>
-      <c r="F17" s="18"/>
-      <c r="G17" s="18"/>
-      <c r="H17" s="19"/>
-      <c r="I17" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J17" s="25"/>
-      <c r="K17" s="26"/>
-    </row>
-    <row r="18" spans="2:11" ht="27" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="22"/>
-      <c r="C18" s="17" t="s">
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="19"/>
+      <c r="K18" s="20"/>
+    </row>
+    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B19" s="12"/>
+      <c r="C19" s="8" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="18"/>
-      <c r="E18" s="18"/>
-      <c r="F18" s="18"/>
-      <c r="G18" s="18"/>
-      <c r="H18" s="19"/>
-      <c r="I18" s="30"/>
-      <c r="J18" s="31"/>
-      <c r="K18" s="32"/>
-    </row>
-    <row r="19" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B19" s="22"/>
-      <c r="C19" s="17" t="s">
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="15"/>
+      <c r="J19" s="19"/>
+      <c r="K19" s="20"/>
+    </row>
+    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B20" s="13"/>
+      <c r="C20" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="18"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="19"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="31"/>
-      <c r="K19" s="32"/>
-    </row>
-    <row r="20" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B20" s="23"/>
-      <c r="C20" s="17" t="s">
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="21"/>
+      <c r="K20" s="22"/>
+    </row>
+    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B21" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="18"/>
-      <c r="E20" s="18"/>
-      <c r="F20" s="18"/>
-      <c r="G20" s="18"/>
-      <c r="H20" s="19"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="28"/>
-      <c r="K20" s="29"/>
-    </row>
-    <row r="21" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B21" s="17" t="s">
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+      <c r="I21" s="9"/>
+      <c r="J21" s="9"/>
+      <c r="K21" s="10"/>
+    </row>
+    <row r="22" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="C21" s="18"/>
-      <c r="D21" s="18"/>
-      <c r="E21" s="18"/>
-      <c r="F21" s="18"/>
-      <c r="G21" s="18"/>
-      <c r="H21" s="18"/>
-      <c r="I21" s="18"/>
-      <c r="J21" s="18"/>
-      <c r="K21" s="19"/>
-    </row>
-    <row r="22" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="21" t="s">
+      <c r="C22" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="C22" s="17" t="s">
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="10"/>
+      <c r="I22" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J22" s="17"/>
+      <c r="K22" s="18"/>
+    </row>
+    <row r="23" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="13"/>
+      <c r="C23" s="8" t="s">
         <v>53</v>
       </c>
-      <c r="D22" s="18"/>
-      <c r="E22" s="18"/>
-      <c r="F22" s="18"/>
-      <c r="G22" s="18"/>
-      <c r="H22" s="19"/>
-      <c r="I22" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J22" s="25"/>
-      <c r="K22" s="26"/>
-    </row>
-    <row r="23" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="23"/>
-      <c r="C23" s="17" t="s">
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="10"/>
+      <c r="I23" s="16"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="22"/>
+    </row>
+    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B24" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="19"/>
-      <c r="I23" s="27"/>
-      <c r="J23" s="28"/>
-      <c r="K23" s="29"/>
-    </row>
-    <row r="24" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B24" s="17" t="s">
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+      <c r="I24" s="9"/>
+      <c r="J24" s="9"/>
+      <c r="K24" s="10"/>
+    </row>
+    <row r="25" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="C24" s="18"/>
-      <c r="D24" s="18"/>
-      <c r="E24" s="18"/>
-      <c r="F24" s="18"/>
-      <c r="G24" s="18"/>
-      <c r="H24" s="18"/>
-      <c r="I24" s="18"/>
-      <c r="J24" s="18"/>
-      <c r="K24" s="19"/>
-    </row>
-    <row r="25" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="21" t="s">
+      <c r="C25" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="C25" s="17" t="s">
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="10"/>
+      <c r="I25" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J25" s="17"/>
+      <c r="K25" s="18"/>
+    </row>
+    <row r="26" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B26" s="13"/>
+      <c r="C26" s="8" t="s">
         <v>57</v>
       </c>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="19"/>
-      <c r="I25" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J25" s="25"/>
-      <c r="K25" s="26"/>
-    </row>
-    <row r="26" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B26" s="23"/>
-      <c r="C26" s="17" t="s">
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="10"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="21"/>
+      <c r="K26" s="22"/>
+    </row>
+    <row r="27" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="D26" s="18"/>
-      <c r="E26" s="18"/>
-      <c r="F26" s="18"/>
-      <c r="G26" s="18"/>
-      <c r="H26" s="19"/>
-      <c r="I26" s="27"/>
-      <c r="J26" s="28"/>
-      <c r="K26" s="29"/>
-    </row>
-    <row r="27" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="33" t="s">
+      <c r="C27" s="8" t="s">
         <v>59</v>
       </c>
-      <c r="C27" s="17" t="s">
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="10"/>
+      <c r="I27" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J27" s="8"/>
+      <c r="K27" s="10"/>
+    </row>
+    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B28" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="D27" s="18"/>
-      <c r="E27" s="18"/>
-      <c r="F27" s="18"/>
-      <c r="G27" s="18"/>
-      <c r="H27" s="19"/>
-      <c r="I27" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J27" s="17"/>
-      <c r="K27" s="19"/>
-    </row>
-    <row r="28" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B28" s="17" t="s">
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+      <c r="I28" s="9"/>
+      <c r="J28" s="9"/>
+      <c r="K28" s="10"/>
+    </row>
+    <row r="29" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="19"/>
-    </row>
-    <row r="29" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="21" t="s">
+      <c r="C29" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C29" s="17" t="s">
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J29" s="17"/>
+      <c r="K29" s="18"/>
+    </row>
+    <row r="30" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="13"/>
+      <c r="C30" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D29" s="18"/>
-      <c r="E29" s="18"/>
-      <c r="F29" s="18"/>
-      <c r="G29" s="18"/>
-      <c r="H29" s="19"/>
-      <c r="I29" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J29" s="25"/>
-      <c r="K29" s="26"/>
-    </row>
-    <row r="30" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="23"/>
-      <c r="C30" s="17" t="s">
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="16"/>
+      <c r="J30" s="21"/>
+      <c r="K30" s="22"/>
+    </row>
+    <row r="31" spans="2:11" x14ac:dyDescent="0.3">
+      <c r="B31" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D30" s="18"/>
-      <c r="E30" s="18"/>
-      <c r="F30" s="18"/>
-      <c r="G30" s="18"/>
-      <c r="H30" s="19"/>
-      <c r="I30" s="27"/>
-      <c r="J30" s="28"/>
-      <c r="K30" s="29"/>
-    </row>
-    <row r="31" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B31" s="17" t="s">
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+      <c r="I31" s="9"/>
+      <c r="J31" s="9"/>
+      <c r="K31" s="10"/>
+    </row>
+    <row r="32" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="C31" s="18"/>
-      <c r="D31" s="18"/>
-      <c r="E31" s="18"/>
-      <c r="F31" s="18"/>
-      <c r="G31" s="18"/>
-      <c r="H31" s="18"/>
-      <c r="I31" s="18"/>
-      <c r="J31" s="18"/>
-      <c r="K31" s="19"/>
-    </row>
-    <row r="32" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="21" t="s">
+      <c r="C32" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="10"/>
+      <c r="I32" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="J32" s="17"/>
+      <c r="K32" s="18"/>
+    </row>
+    <row r="33" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="12"/>
+      <c r="C33" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="18"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="19"/>
-      <c r="I32" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="J32" s="25"/>
-      <c r="K32" s="26"/>
-    </row>
-    <row r="33" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="22"/>
-      <c r="C33" s="17" t="s">
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="10"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="19"/>
+      <c r="K33" s="20"/>
+    </row>
+    <row r="34" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="13"/>
+      <c r="C34" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="18"/>
-      <c r="E33" s="18"/>
-      <c r="F33" s="18"/>
-      <c r="G33" s="18"/>
-      <c r="H33" s="19"/>
-      <c r="I33" s="30"/>
-      <c r="J33" s="31"/>
-      <c r="K33" s="32"/>
-    </row>
-    <row r="34" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="23"/>
-      <c r="C34" s="17" t="s">
+      <c r="D34" s="9"/>
+      <c r="E34" s="9"/>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="10"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="21"/>
+      <c r="K34" s="22"/>
+    </row>
+    <row r="35" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="18"/>
-      <c r="H34" s="19"/>
-      <c r="I34" s="27"/>
-      <c r="J34" s="28"/>
-      <c r="K34" s="29"/>
-    </row>
-    <row r="35" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="17" t="s">
+      <c r="C35" s="9"/>
+      <c r="D35" s="9"/>
+      <c r="E35" s="9"/>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="10"/>
+    </row>
+    <row r="36" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B36" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="C35" s="18"/>
-      <c r="D35" s="18"/>
-      <c r="E35" s="18"/>
-      <c r="F35" s="18"/>
-      <c r="G35" s="18"/>
-      <c r="H35" s="18"/>
-      <c r="I35" s="18"/>
-      <c r="J35" s="18"/>
-      <c r="K35" s="19"/>
-    </row>
-    <row r="36" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="33" t="s">
+      <c r="C36" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="C36" s="17" t="s">
+      <c r="D36" s="9"/>
+      <c r="E36" s="9"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="10"/>
+      <c r="I36" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J36" s="8"/>
+      <c r="K36" s="10"/>
+    </row>
+    <row r="37" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B37" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="19"/>
-      <c r="I36" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J36" s="17"/>
-      <c r="K36" s="19"/>
-    </row>
-    <row r="37" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="33" t="s">
+      <c r="C37" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="C37" s="17" t="s">
+      <c r="D37" s="9"/>
+      <c r="E37" s="9"/>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="10"/>
+      <c r="I37" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="J37" s="8"/>
+      <c r="K37" s="10"/>
+    </row>
+    <row r="38" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
-      <c r="G37" s="18"/>
-      <c r="H37" s="19"/>
-      <c r="I37" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="J37" s="17"/>
-      <c r="K37" s="19"/>
-    </row>
-    <row r="38" spans="2:11" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="34" t="s">
+      <c r="C38" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="C38" s="17" t="s">
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="10"/>
+      <c r="I38" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J38" s="8"/>
+      <c r="K38" s="10"/>
+    </row>
+    <row r="39" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="19"/>
-      <c r="I38" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J38" s="17"/>
-      <c r="K38" s="19"/>
-    </row>
-    <row r="39" spans="2:11" ht="15.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="17" t="s">
+      <c r="C39" s="9"/>
+      <c r="D39" s="9"/>
+      <c r="E39" s="9"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+      <c r="I39" s="9"/>
+      <c r="J39" s="9"/>
+      <c r="K39" s="10"/>
+    </row>
+    <row r="40" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="I39" s="18"/>
-      <c r="J39" s="18"/>
-      <c r="K39" s="19"/>
-    </row>
-    <row r="40" spans="2:11" ht="21" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="33" t="s">
+      <c r="C40" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="C40" s="17" t="s">
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="10"/>
+      <c r="I40" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J40" s="8"/>
+      <c r="K40" s="10"/>
+    </row>
+    <row r="41" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="18"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="19"/>
-      <c r="I40" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J40" s="17"/>
-      <c r="K40" s="19"/>
-    </row>
-    <row r="41" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="33" t="s">
+      <c r="C41" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="C41" s="17" t="s">
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="10"/>
+      <c r="I41" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J41" s="8"/>
+      <c r="K41" s="10"/>
+    </row>
+    <row r="42" spans="2:11" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B42" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="18"/>
-      <c r="H41" s="19"/>
-      <c r="I41" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J41" s="17"/>
-      <c r="K41" s="19"/>
-    </row>
-    <row r="42" spans="2:11" ht="18.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="33" t="s">
+      <c r="C42" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="C42" s="17" t="s">
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="10"/>
+      <c r="I42" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J42" s="8"/>
+      <c r="K42" s="10"/>
+    </row>
+    <row r="43" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="D42" s="18"/>
-      <c r="E42" s="18"/>
-      <c r="F42" s="18"/>
-      <c r="G42" s="18"/>
-      <c r="H42" s="19"/>
-      <c r="I42" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J42" s="17"/>
-      <c r="K42" s="19"/>
-    </row>
-    <row r="43" spans="2:11" ht="28.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="33" t="s">
+      <c r="C43" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="D43" s="9"/>
+      <c r="E43" s="9"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="10"/>
+      <c r="I43" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="J43" s="8"/>
+      <c r="K43" s="10"/>
+    </row>
+    <row r="44" spans="2:11" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B44" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D43" s="18"/>
-      <c r="E43" s="18"/>
-      <c r="F43" s="18"/>
-      <c r="G43" s="18"/>
-      <c r="H43" s="19"/>
-      <c r="I43" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="J43" s="17"/>
-      <c r="K43" s="19"/>
-    </row>
-    <row r="44" spans="2:11" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="C44" s="18"/>
-      <c r="D44" s="18"/>
-      <c r="E44" s="18"/>
-      <c r="F44" s="18"/>
-      <c r="G44" s="18"/>
-      <c r="H44" s="18"/>
-      <c r="I44" s="18"/>
-      <c r="J44" s="18"/>
-      <c r="K44" s="19"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9"/>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" s="9"/>
+      <c r="K44" s="10"/>
     </row>
     <row r="45" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B45" s="1"/>
@@ -2024,6 +2001,79 @@
     <row r="46" spans="2:11" ht="11.1" customHeight="1" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="83">
+    <mergeCell ref="C3:D3"/>
+    <mergeCell ref="G3:H3"/>
+    <mergeCell ref="I3:K3"/>
+    <mergeCell ref="C4:D4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="G5:H5"/>
+    <mergeCell ref="I5:J5"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="I6:K6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="G7:H7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="B8:K8"/>
+    <mergeCell ref="C9:H9"/>
+    <mergeCell ref="J9:K9"/>
+    <mergeCell ref="B10:K10"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="C11:H11"/>
+    <mergeCell ref="J11:K11"/>
+    <mergeCell ref="C12:H12"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="C13:H13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="B14:K14"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:H15"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:K16"/>
+    <mergeCell ref="C16:H16"/>
+    <mergeCell ref="B17:B20"/>
+    <mergeCell ref="C17:H17"/>
+    <mergeCell ref="I17:I20"/>
+    <mergeCell ref="J17:K20"/>
+    <mergeCell ref="C18:H18"/>
+    <mergeCell ref="C19:H19"/>
+    <mergeCell ref="C20:H20"/>
+    <mergeCell ref="B21:K21"/>
+    <mergeCell ref="B22:B23"/>
+    <mergeCell ref="C22:H22"/>
+    <mergeCell ref="I22:I23"/>
+    <mergeCell ref="J22:K23"/>
+    <mergeCell ref="C23:H23"/>
+    <mergeCell ref="B24:K24"/>
+    <mergeCell ref="B25:B26"/>
+    <mergeCell ref="C25:H25"/>
+    <mergeCell ref="I25:I26"/>
+    <mergeCell ref="J25:K26"/>
+    <mergeCell ref="C26:H26"/>
+    <mergeCell ref="C27:H27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="B28:K28"/>
+    <mergeCell ref="B29:B30"/>
+    <mergeCell ref="C29:H29"/>
+    <mergeCell ref="I29:I30"/>
+    <mergeCell ref="J29:K30"/>
+    <mergeCell ref="C30:H30"/>
+    <mergeCell ref="C38:H38"/>
+    <mergeCell ref="J38:K38"/>
+    <mergeCell ref="B31:K31"/>
+    <mergeCell ref="B32:B34"/>
+    <mergeCell ref="C32:H32"/>
+    <mergeCell ref="I32:I34"/>
+    <mergeCell ref="J32:K34"/>
+    <mergeCell ref="C33:H33"/>
+    <mergeCell ref="C34:H34"/>
+    <mergeCell ref="B35:K35"/>
+    <mergeCell ref="C36:H36"/>
+    <mergeCell ref="J36:K36"/>
+    <mergeCell ref="C37:H37"/>
+    <mergeCell ref="J37:K37"/>
     <mergeCell ref="C43:H43"/>
     <mergeCell ref="J43:K43"/>
     <mergeCell ref="B44:K44"/>
@@ -2034,79 +2084,6 @@
     <mergeCell ref="J41:K41"/>
     <mergeCell ref="C42:H42"/>
     <mergeCell ref="J42:K42"/>
-    <mergeCell ref="B35:K35"/>
-    <mergeCell ref="C36:H36"/>
-    <mergeCell ref="J36:K36"/>
-    <mergeCell ref="C37:H37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="C38:H38"/>
-    <mergeCell ref="J38:K38"/>
-    <mergeCell ref="B31:K31"/>
-    <mergeCell ref="B32:B34"/>
-    <mergeCell ref="C32:H32"/>
-    <mergeCell ref="I32:I34"/>
-    <mergeCell ref="J32:K34"/>
-    <mergeCell ref="C33:H33"/>
-    <mergeCell ref="C34:H34"/>
-    <mergeCell ref="C27:H27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="B28:K28"/>
-    <mergeCell ref="B29:B30"/>
-    <mergeCell ref="C29:H29"/>
-    <mergeCell ref="I29:I30"/>
-    <mergeCell ref="J29:K30"/>
-    <mergeCell ref="C30:H30"/>
-    <mergeCell ref="B24:K24"/>
-    <mergeCell ref="B25:B26"/>
-    <mergeCell ref="C25:H25"/>
-    <mergeCell ref="I25:I26"/>
-    <mergeCell ref="J25:K26"/>
-    <mergeCell ref="C26:H26"/>
-    <mergeCell ref="B21:K21"/>
-    <mergeCell ref="B22:B23"/>
-    <mergeCell ref="C22:H22"/>
-    <mergeCell ref="I22:I23"/>
-    <mergeCell ref="J22:K23"/>
-    <mergeCell ref="C23:H23"/>
-    <mergeCell ref="B17:B20"/>
-    <mergeCell ref="C17:H17"/>
-    <mergeCell ref="I17:I20"/>
-    <mergeCell ref="J17:K20"/>
-    <mergeCell ref="C18:H18"/>
-    <mergeCell ref="C19:H19"/>
-    <mergeCell ref="C20:H20"/>
-    <mergeCell ref="B14:K14"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:H15"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:K16"/>
-    <mergeCell ref="C16:H16"/>
-    <mergeCell ref="B10:K10"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="C11:H11"/>
-    <mergeCell ref="J11:K11"/>
-    <mergeCell ref="C12:H12"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="C13:H13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="C7:D7"/>
-    <mergeCell ref="G7:H7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="B8:K8"/>
-    <mergeCell ref="C9:H9"/>
-    <mergeCell ref="J9:K9"/>
-    <mergeCell ref="C5:D5"/>
-    <mergeCell ref="G5:H5"/>
-    <mergeCell ref="I5:J5"/>
-    <mergeCell ref="C6:D6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="C3:D3"/>
-    <mergeCell ref="G3:H3"/>
-    <mergeCell ref="I3:K3"/>
-    <mergeCell ref="C4:D4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="I4:K4"/>
   </mergeCells>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0" right="0" top="0" bottom="0" header="0" footer="0"/>

</xml_diff>